<commit_message>
commit changes on 13th July
</commit_message>
<xml_diff>
--- a/COLLECTION_FRAMEWORK.xlsx
+++ b/COLLECTION_FRAMEWORK.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\MOHAN_PREPARED__JAVA_SQL_NOTE's\prepare_from_office Branch of Java_Interview_Repo\JAVA-INTERVIEW-PREPATAION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{259DFDF3-5DC5-403F-95EE-E47E01CC08C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5872EA17-A7DF-4DC1-8E07-7AC1A3B8B647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="64">
   <si>
     <t>COLLECTION FRAMWORK</t>
   </si>
@@ -160,9 +160,6 @@
   </si>
   <si>
     <t>HashSet with Insetion Order</t>
-  </si>
-  <si>
-    <t>Array of LinkedList (Nodes)</t>
   </si>
   <si>
     <t>INDEX</t>
@@ -261,7 +258,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -292,6 +289,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -458,6 +461,27 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -503,21 +527,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -536,22 +545,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -853,28 +856,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="23.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="25"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="32"/>
     </row>
     <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="43" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="45"/>
+      <c r="A2" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
@@ -902,12 +905,12 @@
     </row>
     <row r="3" spans="1:13" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="B3" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="20" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="16" t="s">
@@ -940,8 +943,8 @@
     </row>
     <row r="4" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="50"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="47"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="21"/>
       <c r="D4" s="16" t="s">
         <v>2</v>
       </c>
@@ -972,8 +975,8 @@
     </row>
     <row r="5" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="50"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="47"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="16" t="s">
         <v>3</v>
       </c>
@@ -1007,7 +1010,7 @@
     </row>
     <row r="6" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="50"/>
-      <c r="B6" s="38"/>
+      <c r="B6" s="25"/>
       <c r="C6" s="48"/>
       <c r="D6" s="16" t="s">
         <v>21</v>
@@ -1039,15 +1042,15 @@
     </row>
     <row r="7" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="50"/>
-      <c r="B7" s="38"/>
-      <c r="C7" s="46" t="s">
+      <c r="B7" s="25"/>
+      <c r="C7" s="20" t="s">
         <v>4</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>5</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="F7" s="5">
         <v>16</v>
@@ -1073,8 +1076,8 @@
     </row>
     <row r="8" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="50"/>
-      <c r="B8" s="38"/>
-      <c r="C8" s="47"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="16" t="s">
         <v>6</v>
       </c>
@@ -1105,13 +1108,13 @@
     </row>
     <row r="9" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="50"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="47"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="16" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>25</v>
@@ -1137,15 +1140,15 @@
     </row>
     <row r="10" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="50"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="46" t="s">
+      <c r="B10" s="25"/>
+      <c r="C10" s="20" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
@@ -1157,13 +1160,13 @@
     </row>
     <row r="11" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="50"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="47"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="21"/>
       <c r="D11" s="16" t="s">
         <v>11</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
@@ -1175,15 +1178,15 @@
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="50"/>
-      <c r="B12" s="37" t="s">
-        <v>50</v>
-      </c>
-      <c r="C12" s="35" t="s">
+      <c r="B12" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="36"/>
+      <c r="D12" s="23"/>
       <c r="E12" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F12" s="11">
         <v>11</v>
@@ -1192,7 +1195,7 @@
         <v>26</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>35</v>
@@ -1207,18 +1210,18 @@
         <v>43</v>
       </c>
       <c r="M12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="50"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="35" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" s="36"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="23"/>
       <c r="E13" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F13" s="11">
         <v>16</v>
@@ -1227,7 +1230,7 @@
         <v>26</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>35</v>
@@ -1242,16 +1245,16 @@
         <v>43</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="50"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="36"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="23"/>
       <c r="E14" s="11" t="s">
         <v>36</v>
       </c>
@@ -1262,7 +1265,7 @@
         <v>26</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>28</v>
@@ -1279,76 +1282,76 @@
     </row>
     <row r="15" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="50"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="E15" s="26" t="s">
+      <c r="B15" s="25"/>
+      <c r="C15" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="42" t="s">
+        <v>55</v>
+      </c>
+      <c r="E15" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="F15" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="I15" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="J15" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="K15" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="F15" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="H15" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="I15" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="J15" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="K15" s="20" t="s">
+      <c r="L15" s="27" t="s">
         <v>61</v>
-      </c>
-      <c r="L15" s="20" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="50"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="28"/>
+      <c r="L16" s="28"/>
     </row>
     <row r="17" spans="1:12" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="51"/>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="29"/>
+      <c r="J17" s="29"/>
+      <c r="K17" s="29"/>
+      <c r="L17" s="29"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="15"/>
       <c r="B20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="18"/>
       <c r="B21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
@@ -1366,11 +1369,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="B12:B17"/>
-    <mergeCell ref="A3:A17"/>
     <mergeCell ref="J15:J17"/>
     <mergeCell ref="K15:K17"/>
     <mergeCell ref="L15:L17"/>
@@ -1387,6 +1385,11 @@
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="B3:B11"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B12:B17"/>
+    <mergeCell ref="A3:A17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>